<commit_message>
feat: add NormalizedAttributes sheet, filter UI CSS
- NormalizedAttributes: ProductID | AttributeGroup | AttributeValue (Step 1 format)
- Filter template: square checkboxes, spacing, cursor UX

Co-authored-by: volodymyr-hohunskyi <volodymyr-hohunskyi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/shared/data/products_import_normalized.xlsx
+++ b/shared/data/products_import_normalized.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="ProductAttributes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ProductFilters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FilterGroups" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Filters" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="NormalizedAttributes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ProductFilters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FilterGroups" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Filters" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -768,17 +769,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>product_id</t>
+          <t>ProductID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>filter_group</t>
+          <t>AttributeGroup</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>filter</t>
+          <t>AttributeValue</t>
         </is>
       </c>
     </row>
@@ -1048,263 +1049,278 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>filter_group_id</t>
+          <t>product_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sort_order</t>
+          <t>filter_group</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>name(en-gb)</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>name(uk-ua)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>name(ru-ru)</t>
+          <t>filter</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
+        <v>101</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Колір</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Цвет</t>
+          <t>Жовтий</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+        <v>101</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cultivation</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Вирощування</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Выращивание</t>
+          <t>Оранжевий</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+        <v>102</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Ріст</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Рост</t>
+          <t>Червоний</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
+        <v>102</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Maturity</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Стиглість</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Спелость</t>
+          <t>Жовтий</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>4</v>
+        <v>102</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Resistance</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Стійкість</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Устойчивость</t>
+          <t>Високорослий</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>5</v>
+        <v>102</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Shape</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Форма</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Форма</t>
+          <t>Розлогий</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>6</v>
+        <v>103</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Texture</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Текстура</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Текстура</t>
+          <t>Рожевий</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
+        <v>103</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Traits</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Особливості</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Особенности</t>
+          <t>Малиновий</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="n">
-        <v>8</v>
+        <v>103</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Вирощування</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Usage</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Призначення</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Назначение</t>
+          <t>Відкритий ґрунт</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="n">
-        <v>9</v>
+        <v>103</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Вирощування</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Yield</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Врожайність</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Урожайность</t>
+          <t>Потребує підв'язки</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>104</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Детермінантний</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>104</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Індетермінантний</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>104</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Вирощування</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Теплиця</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>105</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Жовтий</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>105</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Високорослий</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>105</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Стиглість</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Рання</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>105</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Стиглість</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Середня</t>
         </is>
       </c>
     </row>
@@ -1319,6 +1335,277 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>filter_group_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name(en-gb)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>name(uk-ua)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name(ru-ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Колір</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Цвет</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cultivation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Вирощування</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Выращивание</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ріст</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Maturity</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Стиглість</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Спелость</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Resistance</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Стійкість</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Устойчивость</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Shape</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Форма</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Форма</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Texture</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Текстура</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Текстура</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Traits</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Особливості</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Особенности</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Призначення</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Врожайність</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Урожайность</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>